<commit_message>
update daily dashboard 2026-09-17
</commit_message>
<xml_diff>
--- a/每日输出/石家庄初短/石家庄-石家庄初短-销售风灵在线率明细数据.xlsx
+++ b/每日输出/石家庄初短/石家庄-石家庄初短-销售风灵在线率明细数据.xlsx
@@ -7336,19 +7336,19 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E10" t="n">
         <v>7</v>
       </c>
       <c r="F10" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G10" t="n">
         <v>5</v>
       </c>
       <c r="H10" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="11">
@@ -7364,19 +7364,19 @@
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E11" t="n">
         <v>7</v>
       </c>
       <c r="F11" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G11" t="n">
         <v>5</v>
       </c>
       <c r="H11" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="12">
@@ -7392,19 +7392,19 @@
       </c>
       <c r="C12" t="inlineStr"/>
       <c r="D12" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E12" t="n">
         <v>59</v>
       </c>
       <c r="F12" t="n">
-        <v>0.9365079365079365</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="G12" t="n">
         <v>34</v>
       </c>
       <c r="H12" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.4533333333333333</v>
       </c>
     </row>
   </sheetData>
@@ -7759,19 +7759,19 @@
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E12" s="4" t="n">
         <v>7</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G12" s="4" t="n">
         <v>5</v>
       </c>
       <c r="H12" s="5" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="13">
@@ -7787,19 +7787,19 @@
       </c>
       <c r="C13" s="6" t="inlineStr"/>
       <c r="D13" s="6" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="E13" s="6" t="n">
         <v>7</v>
       </c>
       <c r="F13" s="7" t="n">
-        <v>0.7777777777777778</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="G13" s="6" t="n">
         <v>5</v>
       </c>
       <c r="H13" s="7" t="n">
-        <v>0.5555555555555556</v>
+        <v>0.2380952380952381</v>
       </c>
     </row>
     <row r="14">
@@ -7815,19 +7815,19 @@
       </c>
       <c r="C14" s="6" t="inlineStr"/>
       <c r="D14" s="6" t="n">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="E14" s="6" t="n">
         <v>59</v>
       </c>
       <c r="F14" s="7" t="n">
-        <v>0.9365079365079365</v>
+        <v>0.7866666666666666</v>
       </c>
       <c r="G14" s="6" t="n">
         <v>34</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>0.5396825396825397</v>
+        <v>0.4533333333333333</v>
       </c>
     </row>
   </sheetData>

</xml_diff>